<commit_message>
BA Part 1: Manual artifacts 1, 3, 4 synced with AI content (format kept), N. Boiko removed
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BA/Part 1_Stakeholder Analysis amp Management-20260912/Done/Manual/Artifacts/1. Stakeholder Register_VNS.xlsx
+++ b/BA/Part 1_Stakeholder Analysis amp Management-20260912/Done/Manual/Artifacts/1. Stakeholder Register_VNS.xlsx
@@ -313,7 +313,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -380,6 +380,21 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -733,7 +748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:KH22"/>
+  <dimension ref="A2:KH26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="8.875" customWidth="1" min="1" max="1"/>
@@ -749,7 +764,7 @@
     <col width="38" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="28" customWidth="1" min="13" max="13"/>
-    <col width="18.5" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
     <col width="8.875" customWidth="1" style="3" min="15" max="294"/>
   </cols>
   <sheetData>
@@ -782,7 +797,7 @@
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>"VNS" – Custom University Learning Platform</t>
+          <t>"VNS" — Custom University Learning Platform</t>
         </is>
       </c>
       <c r="D4" s="28" t="n"/>
@@ -796,7 +811,7 @@
       </c>
       <c r="I4" s="29" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="J4" s="28" t="n"/>
@@ -827,7 +842,7 @@
       </c>
       <c r="I5" s="29" t="inlineStr">
         <is>
-          <t>V1.0</t>
+          <t>V1.2</t>
         </is>
       </c>
       <c r="J5" s="28" t="n"/>
@@ -870,7 +885,7 @@
     <row r="7" ht="17.25" customFormat="1" customHeight="1" s="3">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Project Phase </t>
+          <t>Project Phase</t>
         </is>
       </c>
       <c r="C7" s="31" t="inlineStr">
@@ -884,7 +899,7 @@
       <c r="G7" s="28" t="n"/>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Project End Date </t>
+          <t>Project End Date</t>
         </is>
       </c>
       <c r="I7" s="29" t="inlineStr">
@@ -898,7 +913,37 @@
       <c r="M7" s="28" t="n"/>
       <c r="N7" s="28" t="n"/>
     </row>
-    <row r="8" ht="17.25" customFormat="1" customHeight="1" s="3"/>
+    <row r="8" ht="17.25" customFormat="1" customHeight="1" s="3">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>Andrii Lysun (Business Analyst)</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="n"/>
+      <c r="E8" s="28" t="n"/>
+      <c r="F8" s="28" t="n"/>
+      <c r="G8" s="28" t="n"/>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I8" s="29" t="inlineStr">
+        <is>
+          <t>Draft for team approval</t>
+        </is>
+      </c>
+      <c r="J8" s="28" t="n"/>
+      <c r="K8" s="28" t="n"/>
+      <c r="L8" s="28" t="n"/>
+      <c r="M8" s="28" t="n"/>
+      <c r="N8" s="28" t="n"/>
+    </row>
     <row r="9" ht="31.9" customFormat="1" customHeight="1" s="11">
       <c r="B9" s="12" t="inlineStr">
         <is>
@@ -1594,71 +1639,71 @@
       <c r="KG10" s="4" t="n"/>
       <c r="KH10" s="4" t="n"/>
     </row>
-    <row r="11" customFormat="1" s="6">
+    <row r="11" ht="70" customFormat="1" customHeight="1" s="6">
       <c r="A11" s="18" t="n"/>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B11" s="34" t="inlineStr">
         <is>
           <t>Lviv Polytechnic National University</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
-        <is>
-          <t>External/Primary</t>
-        </is>
-      </c>
-      <c r="D11" s="20" t="inlineStr">
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>External / Primary</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="inlineStr">
         <is>
           <t>Key Player</t>
         </is>
       </c>
-      <c r="E11" s="20" t="inlineStr">
+      <c r="E11" s="35" t="inlineStr">
         <is>
           <t>Lviv Polytechnic National University</t>
         </is>
       </c>
-      <c r="F11" s="20" t="inlineStr">
-        <is>
-          <t>Project Sponsor, owner of the future platform</t>
-        </is>
-      </c>
-      <c r="G11" s="20" t="inlineStr">
+      <c r="F11" s="35" t="inlineStr">
+        <is>
+          <t>Project Sponsor — customer and owner of the future platform</t>
+        </is>
+      </c>
+      <c r="G11" s="35" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H11" s="20" t="inlineStr">
+      <c r="H11" s="35" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I11" s="20" t="inlineStr">
-        <is>
-          <t>12 S. Bandery St., Lviv, 79013, Ukraine</t>
-        </is>
-      </c>
-      <c r="J11" s="22" t="inlineStr">
+      <c r="I11" s="35" t="inlineStr">
+        <is>
+          <t>12 S. Bandery Street, Lviv, 79013, Ukraine</t>
+        </is>
+      </c>
+      <c r="J11" s="36" t="inlineStr">
         <is>
           <t>+380 (32) 258-21-11</t>
         </is>
       </c>
-      <c r="K11" s="23" t="inlineStr">
+      <c r="K11" s="37" t="inlineStr">
         <is>
           <t>office@lpnu.ua</t>
         </is>
       </c>
-      <c r="L11" s="20" t="inlineStr">
-        <is>
-          <t>Status meeting + written report</t>
-        </is>
-      </c>
-      <c r="M11" s="20" t="inlineStr">
-        <is>
-          <t>Every second Tuesday</t>
-        </is>
-      </c>
-      <c r="N11" s="21" t="inlineStr">
-        <is>
-          <t>Funds the project, owns the current VNS and the student data, accepts the final result.</t>
+      <c r="L11" s="35" t="inlineStr">
+        <is>
+          <t>Meeting + written status report</t>
+        </is>
+      </c>
+      <c r="M11" s="35" t="inlineStr">
+        <is>
+          <t>Every two weeks, Tuesday</t>
+        </is>
+      </c>
+      <c r="N11" s="38" t="inlineStr">
+        <is>
+          <t>Funds the project, owns the current VNS platform and the student data, and represents the university leadership: approves the project charter and MVP scope and accepts the final result. Main interest is replacing the outdated Moodle-based platform and gaining engagement analytics.</t>
         </is>
       </c>
       <c r="O11" s="3" t="n"/>
@@ -1942,615 +1987,615 @@
       <c r="KG11" s="3" t="n"/>
       <c r="KH11" s="3" t="n"/>
     </row>
-    <row r="12" customFormat="1" s="3">
+    <row r="12" ht="84" customFormat="1" customHeight="1" s="3">
       <c r="A12" s="18" t="n"/>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B12" s="34" t="inlineStr">
         <is>
           <t>Ministry of Education and Science of Ukraine</t>
         </is>
       </c>
-      <c r="C12" s="20" t="inlineStr">
-        <is>
-          <t>External/Secondary</t>
-        </is>
-      </c>
-      <c r="D12" s="20" t="inlineStr">
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>External / Secondary</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>Meet their needs</t>
+        </is>
+      </c>
+      <c r="E12" s="35" t="inlineStr">
+        <is>
+          <t>Ministry of Education and Science of Ukraine</t>
+        </is>
+      </c>
+      <c r="F12" s="35" t="inlineStr">
+        <is>
+          <t>Project Sponsor — sector regulator and funding source</t>
+        </is>
+      </c>
+      <c r="G12" s="35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="35" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I12" s="35" t="inlineStr">
+        <is>
+          <t>10 Peremohy Avenue, Kyiv, 01135, Ukraine</t>
+        </is>
+      </c>
+      <c r="J12" s="36" t="inlineStr">
+        <is>
+          <t>+380 (44) 481-32-21</t>
+        </is>
+      </c>
+      <c r="K12" s="37" t="inlineStr">
+        <is>
+          <t>office@mon.gov.ua</t>
+        </is>
+      </c>
+      <c r="L12" s="35" t="inlineStr">
+        <is>
+          <t>Official one-page report</t>
+        </is>
+      </c>
+      <c r="M12" s="35" t="inlineStr">
+        <is>
+          <t>Once per semester and at control points</t>
+        </is>
+      </c>
+      <c r="N12" s="38" t="inlineStr">
+        <is>
+          <t>Sets the regulatory framework for educational IT systems and for processing personal data in education, and can condition the scaling of the product beyond the pilot. Not involved in day-to-day work: kept satisfied through formal semester reporting and consulted only on decisions with regulatory impact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="98" customFormat="1" customHeight="1" s="3">
+      <c r="A13" s="18" t="n"/>
+      <c r="B13" s="34" t="inlineStr">
+        <is>
+          <t>Technical Department of Lviv Polytechnic</t>
+        </is>
+      </c>
+      <c r="C13" s="35" t="inlineStr">
+        <is>
+          <t>External / Secondary</t>
+        </is>
+      </c>
+      <c r="D13" s="35" t="inlineStr">
         <is>
           <t>Monitor</t>
         </is>
       </c>
-      <c r="E12" s="20" t="inlineStr">
-        <is>
-          <t>Ministry of Education and Science of Ukraine</t>
-        </is>
-      </c>
-      <c r="F12" s="20" t="inlineStr">
-        <is>
-          <t>Sector regulator, formal co-sponsor</t>
-        </is>
-      </c>
-      <c r="G12" s="20" t="inlineStr">
+      <c r="E13" s="35" t="inlineStr">
+        <is>
+          <t>Lviv Polytechnic National University</t>
+        </is>
+      </c>
+      <c r="F13" s="35" t="inlineStr">
+        <is>
+          <t>Developers and administrators of the current VNS</t>
+        </is>
+      </c>
+      <c r="G13" s="35" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H12" s="20" t="inlineStr">
+      <c r="H13" s="35" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I12" s="20" t="inlineStr">
-        <is>
-          <t>10 Peremohy Ave., Kyiv, 01135, Ukraine</t>
-        </is>
-      </c>
-      <c r="J12" s="22" t="inlineStr">
-        <is>
-          <t>+380 (44) 481-32-21</t>
-        </is>
-      </c>
-      <c r="K12" s="23" t="inlineStr">
-        <is>
-          <t>office@mon.gov.ua</t>
-        </is>
-      </c>
-      <c r="L12" s="20" t="inlineStr">
-        <is>
-          <t>No regular communication</t>
-        </is>
-      </c>
-      <c r="M12" s="20" t="inlineStr">
-        <is>
-          <t>Only if regulation changes</t>
-        </is>
-      </c>
-      <c r="N12" s="21" t="inlineStr">
-        <is>
-          <t>No influence on a one-department pilot. Monitored only; no RACI column and no recurring meetings.</t>
+      <c r="I13" s="35" t="inlineStr">
+        <is>
+          <t>12 S. Bandery Street, Lviv, 79013, Ukraine</t>
+        </is>
+      </c>
+      <c r="J13" s="36" t="inlineStr">
+        <is>
+          <t>+380 (32) 258-21-77</t>
+        </is>
+      </c>
+      <c r="K13" s="37" t="inlineStr">
+        <is>
+          <t>it.support@lpnu.ua</t>
+        </is>
+      </c>
+      <c r="L13" s="35" t="inlineStr">
+        <is>
+          <t>E-mail / ticket on request</t>
+        </is>
+      </c>
+      <c r="M13" s="35" t="inlineStr">
+        <is>
+          <t>As needed (registry export, infrastructure access)</t>
+        </is>
+      </c>
+      <c r="N13" s="38" t="inlineStr">
+        <is>
+          <t>Built and maintain the current VNS. Because the project uses its own custom backend with no Moodle integration, the department neither controls delivery nor depends on its result. Involvement is limited to one-off requests: the export of the student registry and access to university infrastructure. Monitored in case they react to the replacement of their system.</t>
         </is>
       </c>
     </row>
-    <row r="13" customFormat="1" s="3">
-      <c r="A13" s="18" t="n"/>
-      <c r="B13" s="19" t="inlineStr">
-        <is>
-          <t>Nataliia Shakhovska</t>
-        </is>
-      </c>
-      <c r="C13" s="20" t="inlineStr">
-        <is>
-          <t>External/Primary</t>
-        </is>
-      </c>
-      <c r="D13" s="19" t="inlineStr">
+    <row r="14" ht="70" customFormat="1" customHeight="1" s="3">
+      <c r="A14" s="18" t="n"/>
+      <c r="B14" s="34" t="inlineStr">
+        <is>
+          <t>End users — students and lecturers</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>External / Primary</t>
+        </is>
+      </c>
+      <c r="D14" s="35" t="inlineStr">
+        <is>
+          <t>Keep Informed</t>
+        </is>
+      </c>
+      <c r="E14" s="35" t="inlineStr">
+        <is>
+          <t>Students and teaching staff of Lviv Polytechnic National University</t>
+        </is>
+      </c>
+      <c r="F14" s="35" t="inlineStr">
+        <is>
+          <t>End users of the product: students and lecturers</t>
+        </is>
+      </c>
+      <c r="G14" s="35" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H14" s="35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I14" s="35" t="inlineStr">
+        <is>
+          <t>12 S. Bandery Street, Lviv, 79013, Ukraine</t>
+        </is>
+      </c>
+      <c r="J14" s="36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K14" s="37" t="inlineStr">
+        <is>
+          <t>Via learning channels and @lpnu.ua mailboxes</t>
+        </is>
+      </c>
+      <c r="L14" s="35" t="inlineStr">
+        <is>
+          <t>Interviews, surveys, usability tests, demos</t>
+        </is>
+      </c>
+      <c r="M14" s="35" t="inlineStr">
+        <is>
+          <t>Weekly during elicitation and the pilot</t>
+        </is>
+      </c>
+      <c r="N14" s="38" t="inlineStr">
+        <is>
+          <t>Primary target audience in two roles. Students: scattered chats, misleading grade summary, empty calendar. Lecturers: course materials, assignments, activity analytics and the AI mode for graded work. No direct influence on decisions, but requirements not validated with them will be wrong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customFormat="1" customHeight="1" s="3">
+      <c r="A15" s="18" t="n"/>
+      <c r="B15" s="34" t="inlineStr">
+        <is>
+          <t>Kostiantyn Holovskyi</t>
+        </is>
+      </c>
+      <c r="C15" s="35" t="inlineStr">
+        <is>
+          <t>Internal / Primary</t>
+        </is>
+      </c>
+      <c r="D15" s="35" t="inlineStr">
+        <is>
+          <t>Key Player</t>
+        </is>
+      </c>
+      <c r="E15" s="35" t="inlineStr">
+        <is>
+          <t>Project team “20/80”</t>
+        </is>
+      </c>
+      <c r="F15" s="35" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="G15" s="35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" s="35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I15" s="35" t="inlineStr">
+        <is>
+          <t>5 Lukasha Street, Lviv, Ukraine</t>
+        </is>
+      </c>
+      <c r="J15" s="36" t="inlineStr">
+        <is>
+          <t>+380 (67) 000-00-01</t>
+        </is>
+      </c>
+      <c r="K15" s="37" t="inlineStr">
+        <is>
+          <t>kostiantyn.holovskyi.shi.2025@lpnu.ua</t>
+        </is>
+      </c>
+      <c r="L15" s="35" t="inlineStr">
+        <is>
+          <t>Team meeting + backlog</t>
+        </is>
+      </c>
+      <c r="M15" s="35" t="inlineStr">
+        <is>
+          <t>Weekly, Monday</t>
+        </is>
+      </c>
+      <c r="N15" s="38" t="inlineStr">
+        <is>
+          <t>Owns the product vision and backlog priorities. Approves the MVP scope and accepts the result from the product side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="70" customFormat="1" customHeight="1" s="3">
+      <c r="A16" s="18" t="n"/>
+      <c r="B16" s="34" t="inlineStr">
+        <is>
+          <t>Nazar Zankovych</t>
+        </is>
+      </c>
+      <c r="C16" s="35" t="inlineStr">
+        <is>
+          <t>Internal / Primary</t>
+        </is>
+      </c>
+      <c r="D16" s="35" t="inlineStr">
         <is>
           <t>Meet their needs</t>
         </is>
       </c>
-      <c r="E13" s="20" t="inlineStr">
-        <is>
-          <t>Rector's Office, Lviv Polytechnic National University</t>
-        </is>
-      </c>
-      <c r="F13" s="19" t="inlineStr">
-        <is>
-          <t>Rector (Executive Sponsor)</t>
-        </is>
-      </c>
-      <c r="G13" s="20" t="inlineStr">
+      <c r="E16" s="35" t="inlineStr">
+        <is>
+          <t>Project team “20/80”</t>
+        </is>
+      </c>
+      <c r="F16" s="35" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="G16" s="35" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H13" s="20" t="inlineStr">
+      <c r="H16" s="35" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I13" s="20" t="inlineStr">
-        <is>
-          <t>12 S. Bandery St., Lviv, 79013, Ukraine</t>
-        </is>
-      </c>
-      <c r="J13" s="22" t="inlineStr">
-        <is>
-          <t>+380 (32) 258-26-00</t>
-        </is>
-      </c>
-      <c r="K13" s="23" t="inlineStr">
-        <is>
-          <t>nataliia.b.shakhovska@lpnu.ua</t>
-        </is>
-      </c>
-      <c r="L13" s="20" t="inlineStr">
-        <is>
-          <t>E-mail with a one-page summary</t>
-        </is>
-      </c>
-      <c r="M13" s="20" t="inlineStr">
-        <is>
-          <t>Once per semester + milestones</t>
-        </is>
-      </c>
-      <c r="N13" s="29" t="inlineStr">
-        <is>
-          <t>Signs the project charter and decides on scaling beyond the pilot. Summary level only.</t>
+      <c r="I16" s="35" t="inlineStr">
+        <is>
+          <t>5 Lukasha Street, Lviv, Ukraine</t>
+        </is>
+      </c>
+      <c r="J16" s="36" t="inlineStr">
+        <is>
+          <t>+380 (67) 000-00-02</t>
+        </is>
+      </c>
+      <c r="K16" s="37" t="inlineStr">
+        <is>
+          <t>nazar.zankovych.shi.2025@lpnu.ua</t>
+        </is>
+      </c>
+      <c r="L16" s="35" t="inlineStr">
+        <is>
+          <t>All project ceremonies</t>
+        </is>
+      </c>
+      <c r="M16" s="35" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="N16" s="38" t="inlineStr">
+        <is>
+          <t>High authority over the plan, schedule, resources and communications. Interest is in delivering on time and within scope rather than in the functional content of the product, which is owned by the Product Owner. Single point of contact for the sponsors.</t>
         </is>
       </c>
     </row>
-    <row r="14" customFormat="1" s="3">
-      <c r="A14" s="18" t="n"/>
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>Nataliia Boiko</t>
-        </is>
-      </c>
-      <c r="C14" s="20" t="inlineStr">
-        <is>
-          <t>External/Primary</t>
-        </is>
-      </c>
-      <c r="D14" s="19" t="inlineStr">
+    <row r="17" ht="42" customFormat="1" customHeight="1" s="3">
+      <c r="A17" s="18" t="n"/>
+      <c r="B17" s="34" t="inlineStr">
+        <is>
+          <t>Andrii Lysun</t>
+        </is>
+      </c>
+      <c r="C17" s="35" t="inlineStr">
+        <is>
+          <t>Internal / Primary</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
         <is>
           <t>Key Player</t>
         </is>
       </c>
-      <c r="E14" s="20" t="inlineStr">
-        <is>
-          <t>Lviv Polytechnic National University</t>
-        </is>
-      </c>
-      <c r="F14" s="19" t="inlineStr">
-        <is>
-          <t>Lecturer – customer and end user</t>
-        </is>
-      </c>
-      <c r="G14" s="20" t="inlineStr">
+      <c r="E17" s="35" t="inlineStr">
+        <is>
+          <t>Project team “20/80”</t>
+        </is>
+      </c>
+      <c r="F17" s="35" t="inlineStr">
+        <is>
+          <t>Business Analyst</t>
+        </is>
+      </c>
+      <c r="G17" s="35" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H14" s="20" t="inlineStr">
+      <c r="H17" s="35" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I14" s="20" t="inlineStr">
-        <is>
-          <t>12 S. Bandery St., Lviv, 79013, Ukraine</t>
-        </is>
-      </c>
-      <c r="J14" s="22" t="inlineStr">
-        <is>
-          <t>+380 (32) 258-25-30</t>
-        </is>
-      </c>
-      <c r="K14" s="23" t="inlineStr">
-        <is>
-          <t>nataliia.i.boiko@lpnu.ua</t>
-        </is>
-      </c>
-      <c r="L14" s="20" t="inlineStr">
-        <is>
-          <t>Interview, workshop, demo</t>
-        </is>
-      </c>
-      <c r="M14" s="20" t="inlineStr">
-        <is>
-          <t>Every Thursday</t>
-        </is>
-      </c>
-      <c r="N14" s="29" t="inlineStr">
-        <is>
-          <t>Defines and accepts the lecturer requirements and will use the product herself.</t>
+      <c r="I17" s="35" t="inlineStr">
+        <is>
+          <t>5 Lukasha Street, Lviv, Ukraine</t>
+        </is>
+      </c>
+      <c r="J17" s="36" t="inlineStr">
+        <is>
+          <t>+380 (67) 000-00-03</t>
+        </is>
+      </c>
+      <c r="K17" s="37" t="inlineStr">
+        <is>
+          <t>andrii.lysun.shi.2025@lpnu.ua</t>
+        </is>
+      </c>
+      <c r="L17" s="35" t="inlineStr">
+        <is>
+          <t>Requirements elicitation meetings, workshops</t>
+        </is>
+      </c>
+      <c r="M17" s="35" t="inlineStr">
+        <is>
+          <t>Weekly + as needed</t>
+        </is>
+      </c>
+      <c r="N17" s="38" t="inlineStr">
+        <is>
+          <t>Elicits and documents requirements and produces the BA artifacts and UML models. Main contact for the end users — both students and lecturers.</t>
         </is>
       </c>
     </row>
-    <row r="15" customFormat="1" s="3">
-      <c r="A15" s="18" t="n"/>
-      <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>Technical Department of Lviv Polytechnic</t>
-        </is>
-      </c>
-      <c r="C15" s="20" t="inlineStr">
-        <is>
-          <t>External/Primary</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
+    <row r="18" ht="56" customFormat="1" customHeight="1" s="3">
+      <c r="A18" s="18" t="n"/>
+      <c r="B18" s="34" t="inlineStr">
+        <is>
+          <t>Denys Lunhul</t>
+        </is>
+      </c>
+      <c r="C18" s="35" t="inlineStr">
+        <is>
+          <t>Internal / Primary</t>
+        </is>
+      </c>
+      <c r="D18" s="35" t="inlineStr">
         <is>
           <t>Key Player</t>
         </is>
       </c>
-      <c r="E15" s="20" t="inlineStr">
-        <is>
-          <t>Lviv Polytechnic National University</t>
-        </is>
-      </c>
-      <c r="F15" s="19" t="inlineStr">
-        <is>
-          <t>Developers and administrators of the current VNS</t>
-        </is>
-      </c>
-      <c r="G15" s="20" t="inlineStr">
+      <c r="E18" s="35" t="inlineStr">
+        <is>
+          <t>Project team “20/80”</t>
+        </is>
+      </c>
+      <c r="F18" s="35" t="inlineStr">
+        <is>
+          <t>Tech Lead, Software Engineer (SWE)</t>
+        </is>
+      </c>
+      <c r="G18" s="35" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H15" s="20" t="inlineStr">
+      <c r="H18" s="35" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I15" s="20" t="inlineStr">
-        <is>
-          <t>12 S. Bandery St., Lviv, 79013, Ukraine</t>
-        </is>
-      </c>
-      <c r="J15" s="22" t="inlineStr">
-        <is>
-          <t>+380 (32) 258-21-77</t>
-        </is>
-      </c>
-      <c r="K15" s="23" t="inlineStr">
-        <is>
-          <t>it.support@lpnu.ua</t>
-        </is>
-      </c>
-      <c r="L15" s="20" t="inlineStr">
-        <is>
-          <t>Working meeting + e-mail</t>
-        </is>
-      </c>
-      <c r="M15" s="20" t="inlineStr">
-        <is>
-          <t>Every two weeks</t>
-        </is>
-      </c>
-      <c r="N15" s="29" t="inlineStr">
-        <is>
-          <t>Own the infrastructure and the student registry. Risk of resistance: engage them as partners.</t>
+      <c r="I18" s="35" t="inlineStr">
+        <is>
+          <t>5 Lukasha Street, Lviv, Ukraine</t>
+        </is>
+      </c>
+      <c r="J18" s="36" t="inlineStr">
+        <is>
+          <t>+380 (67) 000-00-04</t>
+        </is>
+      </c>
+      <c r="K18" s="37" t="inlineStr">
+        <is>
+          <t>denys.lunhul.shi.2025@lpnu.ua</t>
+        </is>
+      </c>
+      <c r="L18" s="35" t="inlineStr">
+        <is>
+          <t>Technical sync + code review</t>
+        </is>
+      </c>
+      <c r="M18" s="35" t="inlineStr">
+        <is>
+          <t>Weekly, Tuesday</t>
+        </is>
+      </c>
+      <c r="N18" s="38" t="inlineStr">
+        <is>
+          <t>Software engineer who also leads the technical side: owns the custom backend architecture, decides on the technology stack and is accountable for the technical feasibility of requirements.</t>
         </is>
       </c>
     </row>
-    <row r="16" customFormat="1" s="3">
-      <c r="A16" s="18" t="n"/>
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>Students of Lviv Polytechnic</t>
-        </is>
-      </c>
-      <c r="C16" s="20" t="inlineStr">
-        <is>
-          <t>External/Primary</t>
-        </is>
-      </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>Keep Informed</t>
-        </is>
-      </c>
-      <c r="E16" s="20" t="inlineStr">
-        <is>
-          <t>Student body of Lviv Polytechnic National University</t>
-        </is>
-      </c>
-      <c r="F16" s="19" t="inlineStr">
-        <is>
-          <t>End users of the platform</t>
-        </is>
-      </c>
-      <c r="G16" s="20" t="inlineStr">
+    <row r="19" ht="84" customFormat="1" customHeight="1" s="3">
+      <c r="A19" s="18" t="n"/>
+      <c r="B19" s="34" t="inlineStr">
+        <is>
+          <t>Yaroslav Shevchuk</t>
+        </is>
+      </c>
+      <c r="C19" s="35" t="inlineStr">
+        <is>
+          <t>Internal / Secondary</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="E19" s="35" t="inlineStr">
+        <is>
+          <t>Project team “20/80”</t>
+        </is>
+      </c>
+      <c r="F19" s="35" t="inlineStr">
+        <is>
+          <t>DevOps, Software Engineer (SWE)</t>
+        </is>
+      </c>
+      <c r="G19" s="35" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H16" s="20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I16" s="20" t="inlineStr">
-        <is>
-          <t>12 S. Bandery St., Lviv, 79013, Ukraine</t>
-        </is>
-      </c>
-      <c r="J16" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K16" s="23" t="inlineStr">
-        <is>
-          <t>via @lpnu.ua mailboxes</t>
-        </is>
-      </c>
-      <c r="L16" s="20" t="inlineStr">
-        <is>
-          <t>Surveys, usability tests</t>
-        </is>
-      </c>
-      <c r="M16" s="20" t="inlineStr">
-        <is>
-          <t>Weekly during the pilot</t>
-        </is>
-      </c>
-      <c r="N16" s="29" t="inlineStr">
-        <is>
-          <t>No say in decisions, but every requirement is validated with them.</t>
+      <c r="H19" s="35" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I19" s="35" t="inlineStr">
+        <is>
+          <t>5 Lukasha Street, Lviv, Ukraine</t>
+        </is>
+      </c>
+      <c r="J19" s="36" t="inlineStr">
+        <is>
+          <t>+380 (67) 000-00-05</t>
+        </is>
+      </c>
+      <c r="K19" s="37" t="inlineStr">
+        <is>
+          <t>yaroslav.shevchuk.shi.2025@lpnu.ua</t>
+        </is>
+      </c>
+      <c r="L19" s="35" t="inlineStr">
+        <is>
+          <t>Daily stand-up + technical sync</t>
+        </is>
+      </c>
+      <c r="M19" s="35" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="N19" s="38" t="inlineStr">
+        <is>
+          <t>Software engineer who also owns deployment, environments and CI/CD. Low influence: executes tasks agreed in planning and does not set scope or priorities. Low interest in the business outcome: engagement is at task level. Kept in the loop through the team's own ceremonies, so no separate stakeholder communication is needed.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="17.25" customFormat="1" customHeight="1" s="3">
-      <c r="A17" s="18" t="n"/>
-      <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>Kostiantyn Holovskyi</t>
-        </is>
-      </c>
-      <c r="C17" s="20" t="inlineStr">
-        <is>
-          <t>Internal/Primary</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>Key Player</t>
-        </is>
-      </c>
-      <c r="E17" s="20" t="inlineStr">
+    <row r="20" ht="70" customFormat="1" customHeight="1" s="5">
+      <c r="A20" s="18" t="n"/>
+      <c r="B20" s="34" t="inlineStr">
+        <is>
+          <t>Volodymyr Kamelchuk</t>
+        </is>
+      </c>
+      <c r="C20" s="35" t="inlineStr">
+        <is>
+          <t>Internal / Secondary</t>
+        </is>
+      </c>
+      <c r="D20" s="35" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="E20" s="35" t="inlineStr">
         <is>
           <t>Project team “20/80”</t>
         </is>
       </c>
-      <c r="F17" s="19" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="G17" s="20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H17" s="20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I17" s="20" t="inlineStr">
-        <is>
-          <t>5 Lukasha St., Lviv, Ukraine</t>
-        </is>
-      </c>
-      <c r="J17" s="22" t="inlineStr">
-        <is>
-          <t>+380 (67) 000-00-01</t>
-        </is>
-      </c>
-      <c r="K17" s="24" t="inlineStr">
-        <is>
-          <t>kostiantyn.holovskyi.shi.2025@lpnu.ua</t>
-        </is>
-      </c>
-      <c r="L17" s="20" t="inlineStr">
-        <is>
-          <t>Planning meeting + backlog</t>
-        </is>
-      </c>
-      <c r="M17" s="20" t="inlineStr">
-        <is>
-          <t>Every Monday</t>
-        </is>
-      </c>
-      <c r="N17" s="29" t="inlineStr">
-        <is>
-          <t>Owns the product vision, the MVP scope and the backlog priorities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" customFormat="1" s="3">
-      <c r="A18" s="18" t="n"/>
-      <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>Nazar Zankovych</t>
-        </is>
-      </c>
-      <c r="C18" s="20" t="inlineStr">
-        <is>
-          <t>Internal/Primary</t>
-        </is>
-      </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>Key Player</t>
-        </is>
-      </c>
-      <c r="E18" s="20" t="inlineStr">
-        <is>
-          <t>Project team “20/80”</t>
-        </is>
-      </c>
-      <c r="F18" s="19" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="G18" s="20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H18" s="20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I18" s="20" t="inlineStr">
-        <is>
-          <t>5 Lukasha St., Lviv, Ukraine</t>
-        </is>
-      </c>
-      <c r="J18" s="22" t="inlineStr">
-        <is>
-          <t>+380 (67) 000-00-02</t>
-        </is>
-      </c>
-      <c r="K18" s="23" t="inlineStr">
-        <is>
-          <t>nazar.zankovych.shi.2025@lpnu.ua</t>
-        </is>
-      </c>
-      <c r="L18" s="20" t="inlineStr">
-        <is>
-          <t>All project meetings</t>
-        </is>
-      </c>
-      <c r="M18" s="20" t="inlineStr">
+      <c r="F20" s="35" t="inlineStr">
+        <is>
+          <t>QA Specialist, Software Engineer (SWE)</t>
+        </is>
+      </c>
+      <c r="G20" s="35" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H20" s="35" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I20" s="35" t="inlineStr">
+        <is>
+          <t>5 Lukasha Street, Lviv, Ukraine</t>
+        </is>
+      </c>
+      <c r="J20" s="36" t="inlineStr">
+        <is>
+          <t>+380 (67) 000-00-06</t>
+        </is>
+      </c>
+      <c r="K20" s="37" t="inlineStr">
+        <is>
+          <t>volodymyr.kamelchuk.shi.2025@lpnu.ua</t>
+        </is>
+      </c>
+      <c r="L20" s="35" t="inlineStr">
+        <is>
+          <t>Daily stand-up + defect report</t>
+        </is>
+      </c>
+      <c r="M20" s="35" t="inlineStr">
         <is>
           <t>Daily</t>
         </is>
       </c>
-      <c r="N18" s="29" t="inlineStr">
-        <is>
-          <t>Plan, schedule, communications; single contact for the sponsors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" customFormat="1" s="3">
-      <c r="A19" s="18" t="n"/>
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>Andrii Lysun</t>
-        </is>
-      </c>
-      <c r="C19" s="20" t="inlineStr">
-        <is>
-          <t>Internal/Primary</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>Key Player</t>
-        </is>
-      </c>
-      <c r="E19" s="20" t="inlineStr">
-        <is>
-          <t>Project team “20/80”</t>
-        </is>
-      </c>
-      <c r="F19" s="19" t="inlineStr">
-        <is>
-          <t>Business Analyst</t>
-        </is>
-      </c>
-      <c r="G19" s="20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H19" s="20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I19" s="20" t="inlineStr">
-        <is>
-          <t>5 Lukasha St., Lviv, Ukraine</t>
-        </is>
-      </c>
-      <c r="J19" s="22" t="inlineStr">
-        <is>
-          <t>+380 (67) 000-00-03</t>
-        </is>
-      </c>
-      <c r="K19" s="23" t="inlineStr">
-        <is>
-          <t>andrii.lysun.shi.2025@lpnu.ua</t>
-        </is>
-      </c>
-      <c r="L19" s="20" t="inlineStr">
-        <is>
-          <t>Elicitation meetings, workshops</t>
-        </is>
-      </c>
-      <c r="M19" s="20" t="inlineStr">
-        <is>
-          <t>Weekly + on demand</t>
-        </is>
-      </c>
-      <c r="N19" s="29" t="inlineStr">
-        <is>
-          <t>Elicits and documents requirements, owns the BA artifacts and UML models.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" customFormat="1" s="5">
-      <c r="A20" s="18" t="n"/>
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>Denys Lunhul</t>
-        </is>
-      </c>
-      <c r="C20" s="20" t="inlineStr">
-        <is>
-          <t>Internal/Primary</t>
-        </is>
-      </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>Key Player</t>
-        </is>
-      </c>
-      <c r="E20" s="20" t="inlineStr">
-        <is>
-          <t>Project team “20/80”</t>
-        </is>
-      </c>
-      <c r="F20" s="19" t="inlineStr">
-        <is>
-          <t>Tech Lead</t>
-        </is>
-      </c>
-      <c r="G20" s="20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H20" s="20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I20" s="20" t="inlineStr">
-        <is>
-          <t>5 Lukasha St., Lviv, Ukraine</t>
-        </is>
-      </c>
-      <c r="J20" s="22" t="inlineStr">
-        <is>
-          <t>+380 (67) 000-00-04</t>
-        </is>
-      </c>
-      <c r="K20" s="23" t="inlineStr">
-        <is>
-          <t>denys.lunhul.shi.2025@lpnu.ua</t>
-        </is>
-      </c>
-      <c r="L20" s="20" t="inlineStr">
-        <is>
-          <t>Technical sync + code review</t>
-        </is>
-      </c>
-      <c r="M20" s="20" t="inlineStr">
-        <is>
-          <t>Every Tuesday</t>
-        </is>
-      </c>
-      <c r="N20" s="29" t="inlineStr">
-        <is>
-          <t>Backend architecture, data model and technology stack decisions.</t>
+      <c r="N20" s="38" t="inlineStr">
+        <is>
+          <t>Software engineer who also verifies the acceptance criteria, in particular the grade forecast and the AI's refusal to produce complete solutions for graded work. Low influence and low interest in the business outcome; kept in the loop through the team's own ceremonies.</t>
         </is>
       </c>
       <c r="O20" s="3" t="n"/>
@@ -2836,146 +2881,121 @@
     </row>
     <row r="21" customFormat="1" s="3">
       <c r="A21" s="18" t="n"/>
-      <c r="B21" s="19" t="inlineStr">
-        <is>
-          <t>Yaroslav Shevchuk</t>
-        </is>
-      </c>
-      <c r="C21" s="20" t="inlineStr">
-        <is>
-          <t>Internal/Secondary</t>
-        </is>
-      </c>
-      <c r="D21" s="19" t="inlineStr">
-        <is>
-          <t>Keep Informed</t>
-        </is>
-      </c>
-      <c r="E21" s="20" t="inlineStr">
-        <is>
-          <t>Project team “20/80”</t>
-        </is>
-      </c>
-      <c r="F21" s="19" t="inlineStr">
-        <is>
-          <t>DevOps</t>
-        </is>
-      </c>
-      <c r="G21" s="20" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H21" s="20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I21" s="20" t="inlineStr">
-        <is>
-          <t>5 Lukasha St., Lviv, Ukraine</t>
-        </is>
-      </c>
-      <c r="J21" s="22" t="inlineStr">
-        <is>
-          <t>+380 (67) 000-00-05</t>
-        </is>
-      </c>
-      <c r="K21" s="23" t="inlineStr">
-        <is>
-          <t>yaroslav.shevchuk.shi.2025@lpnu.ua</t>
-        </is>
-      </c>
-      <c r="L21" s="20" t="inlineStr">
-        <is>
-          <t>Daily stand-up</t>
-        </is>
-      </c>
-      <c r="M21" s="20" t="inlineStr">
-        <is>
-          <t>Daily</t>
-        </is>
-      </c>
-      <c r="N21" s="29" t="inlineStr">
-        <is>
-          <t>Environments, CI/CD and workers for AI tasks; works with the Tech Department.</t>
-        </is>
-      </c>
       <c r="O21" s="3" t="n"/>
     </row>
     <row r="22" customFormat="1" s="3">
       <c r="A22" s="18" t="n"/>
-      <c r="B22" s="19" t="inlineStr">
-        <is>
-          <t>Volodymyr Kamelchuk</t>
-        </is>
-      </c>
-      <c r="C22" s="20" t="inlineStr">
-        <is>
-          <t>Internal/Secondary</t>
-        </is>
-      </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>Keep Informed</t>
-        </is>
-      </c>
-      <c r="E22" s="20" t="inlineStr">
-        <is>
-          <t>Project team “20/80”</t>
-        </is>
-      </c>
-      <c r="F22" s="19" t="inlineStr">
-        <is>
-          <t>QA Specialist</t>
-        </is>
-      </c>
-      <c r="G22" s="20" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H22" s="20" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I22" s="20" t="inlineStr">
-        <is>
-          <t>5 Lukasha St., Lviv, Ukraine</t>
-        </is>
-      </c>
-      <c r="J22" s="22" t="inlineStr">
-        <is>
-          <t>+380 (67) 000-00-06</t>
-        </is>
-      </c>
-      <c r="K22" s="23" t="inlineStr">
-        <is>
-          <t>volodymyr.kamelchuk.shi.2025@lpnu.ua</t>
-        </is>
-      </c>
-      <c r="L22" s="20" t="inlineStr">
-        <is>
-          <t>Daily stand-up + defect report</t>
-        </is>
-      </c>
-      <c r="M22" s="20" t="inlineStr">
-        <is>
-          <t>Daily</t>
-        </is>
-      </c>
-      <c r="N22" s="29" t="inlineStr">
-        <is>
-          <t>Checks acceptance criteria, the grade forecast and the AI refusal rules.</t>
-        </is>
-      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>LEGEND AND COMPLETION RULES</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="n"/>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="12" t="n"/>
+      <c r="G22" s="12" t="n"/>
+      <c r="H22" s="12" t="n"/>
+      <c r="I22" s="12" t="n"/>
+      <c r="J22" s="12" t="n"/>
+      <c r="K22" s="12" t="n"/>
+      <c r="L22" s="12" t="n"/>
+      <c r="M22" s="12" t="n"/>
+      <c r="N22" s="12" t="n"/>
       <c r="O22" s="3" t="n"/>
     </row>
-    <row r="23" customFormat="1" s="3"/>
-    <row r="24" customFormat="1" s="3"/>
-    <row r="25" customFormat="1" s="3"/>
-    <row r="26" customFormat="1" s="3"/>
+    <row r="23" ht="17.25" customFormat="1" customHeight="1" s="3">
+      <c r="B23" s="34" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C23" s="35" t="inlineStr">
+        <is>
+          <t>Internal — a member of the delivery team; External — a stakeholder on the university or state side. Primary — directly involved; Secondary — involved indirectly.</t>
+        </is>
+      </c>
+      <c r="D23" s="35" t="n"/>
+      <c r="E23" s="35" t="n"/>
+      <c r="F23" s="35" t="n"/>
+      <c r="G23" s="35" t="n"/>
+      <c r="H23" s="35" t="n"/>
+      <c r="I23" s="35" t="n"/>
+      <c r="J23" s="36" t="n"/>
+      <c r="K23" s="37" t="n"/>
+      <c r="L23" s="35" t="n"/>
+      <c r="M23" s="35" t="n"/>
+      <c r="N23" s="38" t="n"/>
+    </row>
+    <row r="24" ht="17.25" customFormat="1" customHeight="1" s="3">
+      <c r="B24" s="34" t="inlineStr">
+        <is>
+          <t>Stakeholder Group</t>
+        </is>
+      </c>
+      <c r="C24" s="35" t="inlineStr">
+        <is>
+          <t>Derived from Power/Influence × Interest: High+High = Key Player (ENGAGE); High+Low = Meet their needs (SATISFY); Low+High = Keep Informed (INFORM); Low+Low = Monitor (MONITOR).</t>
+        </is>
+      </c>
+      <c r="D24" s="35" t="n"/>
+      <c r="E24" s="35" t="n"/>
+      <c r="F24" s="35" t="n"/>
+      <c r="G24" s="35" t="n"/>
+      <c r="H24" s="35" t="n"/>
+      <c r="I24" s="35" t="n"/>
+      <c r="J24" s="36" t="n"/>
+      <c r="K24" s="37" t="n"/>
+      <c r="L24" s="35" t="n"/>
+      <c r="M24" s="35" t="n"/>
+      <c r="N24" s="38" t="n"/>
+    </row>
+    <row r="25" ht="28" customFormat="1" customHeight="1" s="3">
+      <c r="B25" s="34" t="inlineStr">
+        <is>
+          <t>MONITOR quadrant</t>
+        </is>
+      </c>
+      <c r="C25" s="35" t="inlineStr">
+        <is>
+          <t>The Technical Department, DevOps and QA sit here. The department only handles one-off requests because the custom backend does not depend on the current VNS; DevOps and QA execute agreed tasks and are kept in the loop through the team's own ceremonies.</t>
+        </is>
+      </c>
+      <c r="D25" s="35" t="n"/>
+      <c r="E25" s="35" t="n"/>
+      <c r="F25" s="35" t="n"/>
+      <c r="G25" s="35" t="n"/>
+      <c r="H25" s="35" t="n"/>
+      <c r="I25" s="35" t="n"/>
+      <c r="J25" s="36" t="n"/>
+      <c r="K25" s="37" t="n"/>
+      <c r="L25" s="35" t="n"/>
+      <c r="M25" s="35" t="n"/>
+      <c r="N25" s="38" t="n"/>
+    </row>
+    <row r="26" ht="17.25" customFormat="1" customHeight="1" s="3">
+      <c r="B26" s="34" t="inlineStr">
+        <is>
+          <t>Contact details</t>
+        </is>
+      </c>
+      <c r="C26" s="35" t="inlineStr">
+        <is>
+          <t>Phone numbers are illustrative placeholders for this training project. Team e-mail addresses follow the real Lviv Polytechnic National University format.</t>
+        </is>
+      </c>
+      <c r="D26" s="35" t="n"/>
+      <c r="E26" s="35" t="n"/>
+      <c r="F26" s="35" t="n"/>
+      <c r="G26" s="35" t="n"/>
+      <c r="H26" s="35" t="n"/>
+      <c r="I26" s="35" t="n"/>
+      <c r="J26" s="36" t="n"/>
+      <c r="K26" s="37" t="n"/>
+      <c r="L26" s="35" t="n"/>
+      <c r="M26" s="35" t="n"/>
+      <c r="N26" s="38" t="n"/>
+    </row>
     <row r="27" customFormat="1" s="3"/>
     <row r="28" customFormat="1" s="3"/>
     <row r="29" customFormat="1" s="3"/>
@@ -3006,13 +3026,20 @@
     <row r="54" customFormat="1" s="3"/>
     <row r="55" customFormat="1" s="3"/>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="16">
     <mergeCell ref="I7:N7"/>
+    <mergeCell ref="C8:G8"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="C4:G4"/>
+    <mergeCell ref="B22:N22"/>
+    <mergeCell ref="C24:N24"/>
     <mergeCell ref="C6:G6"/>
     <mergeCell ref="I5:N5"/>
+    <mergeCell ref="C25:N25"/>
+    <mergeCell ref="C23:N23"/>
     <mergeCell ref="C5:G5"/>
+    <mergeCell ref="I8:N8"/>
+    <mergeCell ref="C26:N26"/>
     <mergeCell ref="I4:N4"/>
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="I6:N6"/>

</xml_diff>